<commit_message>
Added shortcut to center window Ctrl+Shift+C
</commit_message>
<xml_diff>
--- a/inputs/buttons.xlsx
+++ b/inputs/buttons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tuan\Documents\GitHub\tuans_world\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307C589D-13FC-4C1C-BA9F-FB4554FD6A89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{823B9A71-A8C9-464C-A0C1-EC5746903E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="3090" windowWidth="21600" windowHeight="11295" xr2:uid="{F53843A5-4C8D-4DE0-AFBD-DDF1A7BEE99F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F53843A5-4C8D-4DE0-AFBD-DDF1A7BEE99F}"/>
   </bookViews>
   <sheets>
     <sheet name="Buttons" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="29">
   <si>
     <t>Button</t>
   </si>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <t>C:\Users\tuan\Anaconda3\envs\icrm\Scripts\designer.exe</t>
+  </si>
+  <si>
+    <t>Pictures</t>
+  </si>
+  <si>
+    <t>C:\Users\tuan\Documents</t>
   </si>
 </sst>
 </file>
@@ -466,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56BAA9C9-76B0-469F-9CFA-41DD7A7485DD}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
@@ -656,6 +662,20 @@
         <v>23</v>
       </c>
     </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>